<commit_message>
final update week 19
</commit_message>
<xml_diff>
--- a/rates-nodispo/week-19/Analisis_Rates_NoDispo_7d.xlsx
+++ b/rates-nodispo/week-19/Analisis_Rates_NoDispo_7d.xlsx
@@ -570,7 +570,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -5690,7 +5690,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8043,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -9886,7 +9886,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -14477,7 +14477,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -14630,7 +14630,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -14783,7 +14783,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -14944,7 +14944,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -17552,7 +17552,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -19597,7 +19597,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -21950,7 +21950,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -23793,7 +23793,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -25636,7 +25636,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -28769,7 +28769,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -28922,7 +28922,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -29083,7 +29083,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -31691,7 +31691,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -33737,7 +33737,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -36247,7 +36247,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -38600,7 +38600,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -40443,7 +40443,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -42286,7 +42286,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -45951,7 +45951,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -48303,7 +48303,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -50192,7 +50192,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -52191,7 +52191,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -54190,7 +54190,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -56186,7 +56186,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11/05/2026 15:07 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 11/05/2026 17:43 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>